<commit_message>
adding gitignore and updating conversion examples from the paper
</commit_message>
<xml_diff>
--- a/paper_examples_converted.xlsx
+++ b/paper_examples_converted.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bmeyers/github/deanthro/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FDE7CA0-4127-114E-874F-955AF6D11AD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8F84E93-C59A-A847-A272-A6CF433AE291}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{29A44382-B293-A74B-8E54-729C68D5C14B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t>Input</t>
   </si>
@@ -414,6 +414,51 @@
 - **User-centric framing** – Shifts focus to human perception, not machine intent.  
 - **Precise language** – Uses terms like "configured," "responses," and "perceive" to describe observable facts.  
 This aligns with the principle that systems simulate—rather than experience—interpersonal dynamics.</t>
+  </si>
+  <si>
+    <t>Here’s the de-anthropomorphized version:  
+**"Early-stage conversational systems [...] have constrained functionality for"**  
+### Key Changes:  
+1. **"chatbot"** → **"conversational system"**  
+   - Removes the personified "-bot" suffix in favor of a technical descriptor.  
+2. **"prototypes"** → **"early-stage"**  
+   - More precise (not all prototypes are early-stage, and vice versa).  
+3. **"limited capability of"** → **"constrained functionality for"**  
+   - "Capability" implies potential agency; "functionality" describes designed features.  
+### Alternative Phrasing:  
+- *"Experimental text-based interfaces [...] operate within narrow parameters for"*  
+- *"Pilot dialogue systems [...] are restricted to handling"*  
+### Why This Works:  
+- **No implied agency** – Focuses on system *design* (what it’s built to do) rather than *abilities* (what it "can" do).  
+- **Technical accuracy** – "Constrained functionality" reflects engineering limits, not cognitive limits.  
+- **Scalability** – Works for any automated system, avoiding anthropomorphic metaphors.  
+This aligns with the framework’s goal of describing systems as tools, not agents.</t>
+  </si>
+  <si>
+    <t>“chat simulator prototypes […] have limited functionality for”</t>
+  </si>
+  <si>
+    <t>Here's the de-anthropomorphized version:
+"chat simulator prototypes [...] have limited functionality for"
+**Changes made:**
+- "chatbot" → "chat simulator" (standard substitution for communication category)
+- "capability of" → "functionality for" (removes "products of cognition" term, emphasizes what the system does rather than what it "can do")
+**Alternative versions:**
+"chat simulator prototypes [...] are limited in their ability to"
+- Still focuses on functional limitations
+- Slightly different phrasing
+"these text generation systems [...] have constraints in"
+- Emphasizes the constraints/boundaries
+- Uses "systems" for variety
+**User-focused alternative:**
+"users of chat simulator prototypes [...] have limited ability to"
+- Relocates the limitation to what users can do with the system
+- Maintains focus on human agency
+**Technical alternative:**
+"chat simulator prototypes [...] produce limited output types for"
+- Most specific about what's actually limited
+- Describes the output characteristics
+The key issue: "capability" is a products of cognition term—it implies skills or abilities gained through learning/intelligence. Systems have functionalities, features, or operational parameters, not capabilities in the cognitive sense.</t>
   </si>
 </sst>
 </file>
@@ -462,7 +507,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -470,8 +515,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -811,218 +862,248 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
-    <col min="2" max="5" width="50.83203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="50.83203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="75.83203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="50.83203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="75.83203125" style="1" customWidth="1"/>
     <col min="6" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="2" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="1">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A3" s="1">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="4" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A4" s="1">
+      <c r="A4" s="4">
         <v>1</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="4" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
+      <c r="A5" s="4">
         <v>1</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="4" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
+      <c r="A6" s="4">
         <v>1</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
+      <c r="A7" s="4">
         <v>2</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" s="4" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A8" s="1">
+      <c r="A8" s="4">
         <v>2</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" s="4" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A9" s="1">
+      <c r="A9" s="4">
         <v>2</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="4" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A10" s="1">
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+    </row>
+    <row r="10" spans="1:5" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A10" s="4">
         <v>2</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="4" t="s">
         <v>31</v>
       </c>
+      <c r="C10" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="11" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A11" s="1">
+      <c r="A11" s="4">
         <v>2</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="4" t="s">
         <v>32</v>
       </c>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
     </row>
     <row r="12" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A12" s="1">
+      <c r="A12" s="4">
         <v>3</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="4" t="s">
         <v>33</v>
       </c>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
     </row>
     <row r="13" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A13" s="1">
+      <c r="A13" s="4">
         <v>3</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="4" t="s">
         <v>34</v>
       </c>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
     </row>
     <row r="14" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A14" s="1">
+      <c r="A14" s="4">
         <v>3</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="4" t="s">
         <v>35</v>
       </c>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
     </row>
     <row r="15" spans="1:5" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A15" s="1">
+      <c r="A15" s="4">
         <v>3</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="D15" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="E15" s="4" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A16" s="1">
+      <c r="A16" s="4">
         <v>3</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="4" t="s">
         <v>37</v>
       </c>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>